<commit_message>
vault backup: 2026-10-23 19:06:28
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-10-23.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-10-23.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -529,27 +529,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건강-20261019-001</t>
+          <t>경영-20261023-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>신민경</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -557,25 +557,25 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>카페24</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>네이버 SA&amp;GFA 광고 비용</t>
+          <t>sms 충전 비용</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>2948000</v>
+        <v>1500000</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>미정</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -585,61 +585,56 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>10/20(화)~10/21(수) 광고비</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>건강-20261019-004</t>
+          <t>경영-20261023-003</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ADN</t>
+          <t>부가세</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ADN 배너 광고 비용</t>
+          <t>2기 예정 부가세</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>550000</v>
+        <v>27948150</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -653,29 +648,34 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>세금·보험(대외비)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>건강-20261019-006</t>
+          <t>경영-20261019-010</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -684,46 +684,51 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>비오템</t>
+          <t>농협카드</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>10월브스라이브경품(튼살크림)</t>
+          <t>카드대금</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>70000</v>
+        <v>4973743</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>미정</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>변경</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>경영-20261019-001</t>
+          <t>경영-20261023-002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -738,38 +743,43 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김솔이</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>이앤씨이노비즈타워</t>
+          <t>카페24</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>본사 9월 관리비 납부</t>
+          <t>카페24 sms충전</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1569060</v>
+        <v>1000000</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>법인카드</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>우리카드</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -779,19 +789,14 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>에이팜</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>경영-20261019-008</t>
+          <t>경영-20261023-004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -811,29 +816,29 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>대청하이츠</t>
+          <t>남경 노무법인</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>기숙사 월세 및 관리비</t>
+          <t>인사자문수수료</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>350000</v>
+        <v>275000</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -847,7 +852,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -859,49 +864,49 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건강-20261019-007</t>
+          <t>데이터-20261023-001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>데이터</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>데이터사이언스팀</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>조성윤</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>엘앤에이치컴퍼니</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>10월브스라이브구매인증(적립금)</t>
+          <t>사무실 임대비용</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>30000</v>
+        <v>1650000</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -915,56 +920,56 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>건강-20261019-002</t>
+          <t>물류-20261023-001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>물류</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>물류팀</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>허수원</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>(주)한진택배</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>네이버 SA&amp;GFA 광고 비용</t>
+          <t>9월 에이팜 한진택배비</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2728000</v>
+        <v>68200</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -978,61 +983,61 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/22(목)~10/23(금) 광고비</t>
+          <t>에이팜</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>건강-20261019-011</t>
+          <t>물류-20261023-002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>물류</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>물류팀</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>허수원</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>원정대</t>
+          <t>(주)한진택배</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>9월 META 광고 대행 수수료</t>
+          <t>9월 에이팜건강 한진택배비</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>298398</v>
+        <v>8563720</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1046,124 +1051,129 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>에이팜건강</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>경영-20261021-001</t>
+          <t>건강-20261019-005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>장은총</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>15그램</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>영상 제작 및 체험단</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>11220000</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>계좌송금</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>변경</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>개별지급(허수원, 장은총, 김정원, 류기련)</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>워크샵 유류비&amp;주차비용</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>52000</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>계좌송금</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>1인당 13,000원</t>
+          <t>700만원 페이백 예정 (11월~12월 중)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강-20261019-008</t>
+          <t>경영-20261023-005</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>에이팜</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>네이버톡톡</t>
+          <t>이동매출</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>500000</v>
+        <v>111197</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1177,56 +1187,61 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>건강-20261019-003</t>
+          <t>경영-20261023-006</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>서원회계법인</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>네이버 SA&amp;GFA 광고 비용</t>
+          <t>기장료</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>4422000</v>
+        <v>385000</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1240,65 +1255,70 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>10/24(토)~10/26(월) 광고비</t>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>건강-20261019-009</t>
+          <t>경영-20261023-007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>한국건강기능식품협회</t>
+          <t>쿠팡</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>11월 1차 라이브 심의</t>
+          <t>직원 간식</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>400000</v>
+        <v>370000</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>법인카드</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>우리카드</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1308,219 +1328,10 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>예상금액으로 달라질 수 있음(제품컨펌 아직X)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>경영-20261019-002</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>경영</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>경영지원팀</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>송채은</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>비씨카드</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>비씨카드 대금 지출건 (9월)</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>1346060</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>자동이체</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>에이팜</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>경영-20261019-009</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>경영</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>경영지원팀</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>김수희</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>9</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>사구플라워</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>대표님 지인(정찬용) 결혼 축하화환</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>49000</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>법인카드</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>우리카드</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>경영-20261019-011</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>경영</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>경영지원팀</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>김수희</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>11</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>우리카드</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>카드대금</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>29462497</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>자동이체</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>기타 대외비 지출</t>
         </is>

</xml_diff>